<commit_message>
Update dexa trust names
</commit_message>
<xml_diff>
--- a/Data/National-Imaging-Data-Collection-Asset-Count-2022-23-v1.xlsx
+++ b/Data/National-Imaging-Data-Collection-Asset-Count-2022-23-v1.xlsx
@@ -1,22 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26924"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nhsengland.sharepoint.com/sites/CFO/ofp/pat/Restricted document/UEC &amp; AP/Diagnostics/NIDC/Publication/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://healthsharedservice-my.sharepoint.com/personal/anne_foulger_dhsc_gov_uk/Documents/repos/FLS_mapping/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="76" documentId="8_{FDCA17FA-C2FF-442C-91F5-FF17B8E5D6A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5A47A523-A460-41F7-9BE0-D04B7DCA852E}"/>
+  <xr:revisionPtr revIDLastSave="81" documentId="8_{FDCA17FA-C2FF-442C-91F5-FF17B8E5D6A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{062A8A50-63FA-4F43-B389-2E7D45DCF412}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{79F2D076-C940-4B30-8FDD-1AECEE309C4D}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="19200" windowHeight="10060" activeTab="2" xr2:uid="{79F2D076-C940-4B30-8FDD-1AECEE309C4D}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="21" r:id="rId1"/>
     <sheet name="England and Regional" sheetId="22" r:id="rId2"/>
     <sheet name="ICB, Imaging Network and Trust" sheetId="1" r:id="rId3"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'ICB, Imaging Network and Trust'!$A$14:$V$151</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -1799,15 +1802,15 @@
     <xf numFmtId="0" fontId="26" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="14" fillId="6" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="14" fillId="6" borderId="8" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1886,9 +1889,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1926,7 +1929,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -2032,7 +2035,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2174,7 +2177,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -2183,19 +2186,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA835F15-C7B1-49E4-B38C-5A7B4039B0E7}">
   <dimension ref="B2:G33"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.08984375" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="2.109375" style="18" customWidth="1"/>
-    <col min="2" max="2" width="28.88671875" style="18" customWidth="1"/>
-    <col min="3" max="3" width="33.5546875" style="18" customWidth="1"/>
-    <col min="4" max="4" width="59.88671875" style="18" customWidth="1"/>
+    <col min="1" max="1" width="2.08984375" style="18" customWidth="1"/>
+    <col min="2" max="2" width="28.90625" style="18" customWidth="1"/>
+    <col min="3" max="3" width="33.54296875" style="18" customWidth="1"/>
+    <col min="4" max="4" width="59.90625" style="18" customWidth="1"/>
     <col min="5" max="5" width="42" style="18" customWidth="1"/>
-    <col min="6" max="12" width="6.88671875" style="18" customWidth="1"/>
-    <col min="13" max="16384" width="9.109375" style="18"/>
+    <col min="6" max="12" width="6.90625" style="18" customWidth="1"/>
+    <col min="13" max="16384" width="9.08984375" style="18"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:7" ht="6" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="3" spans="2:7" ht="35.4" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:7" ht="6" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="3" spans="2:7" ht="35" x14ac:dyDescent="0.35">
       <c r="B3" s="62" t="s">
         <v>67</v>
       </c>
@@ -2203,7 +2206,7 @@
       <c r="D3" s="63"/>
       <c r="E3" s="63"/>
     </row>
-    <row r="5" spans="2:7" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:7" ht="18" x14ac:dyDescent="0.4">
       <c r="B5" s="19" t="s">
         <v>52</v>
       </c>
@@ -2211,7 +2214,7 @@
       <c r="D5" s="20"/>
       <c r="E5" s="20"/>
     </row>
-    <row r="6" spans="2:7" ht="95.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:7" ht="95.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B6" s="64" t="s">
         <v>404</v>
       </c>
@@ -2220,7 +2223,7 @@
       <c r="E6" s="65"/>
       <c r="G6" s="22"/>
     </row>
-    <row r="7" spans="2:7" ht="31.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:7" ht="31.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B7" s="19" t="s">
         <v>53</v>
       </c>
@@ -2228,7 +2231,7 @@
       <c r="D7" s="21"/>
       <c r="E7" s="21"/>
     </row>
-    <row r="8" spans="2:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:7" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B8" s="40" t="s">
         <v>342</v>
       </c>
@@ -2236,7 +2239,7 @@
       <c r="D8" s="21"/>
       <c r="E8" s="21"/>
     </row>
-    <row r="9" spans="2:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:7" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B9" s="40" t="s">
         <v>350</v>
       </c>
@@ -2244,7 +2247,7 @@
       <c r="D9" s="21"/>
       <c r="E9" s="21"/>
     </row>
-    <row r="10" spans="2:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:7" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B10" s="40" t="s">
         <v>343</v>
       </c>
@@ -2252,20 +2255,20 @@
       <c r="D10" s="21"/>
       <c r="E10" s="21"/>
     </row>
-    <row r="11" spans="2:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:7" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B11" s="23"/>
       <c r="C11" s="21"/>
       <c r="D11" s="21"/>
       <c r="E11" s="21"/>
     </row>
-    <row r="12" spans="2:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:7" ht="15.5" x14ac:dyDescent="0.35">
       <c r="C12" s="50" t="s">
         <v>352</v>
       </c>
       <c r="D12" s="21"/>
       <c r="E12" s="21"/>
     </row>
-    <row r="13" spans="2:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:7" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B13" s="24" t="s">
         <v>61</v>
       </c>
@@ -2275,7 +2278,7 @@
       <c r="D13" s="21"/>
       <c r="E13" s="21"/>
     </row>
-    <row r="14" spans="2:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:7" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B14" s="24" t="s">
         <v>62</v>
       </c>
@@ -2285,7 +2288,7 @@
       <c r="D14" s="21"/>
       <c r="E14" s="21"/>
     </row>
-    <row r="15" spans="2:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:7" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B15" s="59" t="s">
         <v>338</v>
       </c>
@@ -2295,7 +2298,7 @@
       <c r="D15" s="21"/>
       <c r="E15" s="21"/>
     </row>
-    <row r="16" spans="2:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:7" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B16" s="61"/>
       <c r="C16" s="46" t="s">
         <v>347</v>
@@ -2303,7 +2306,7 @@
       <c r="D16" s="21"/>
       <c r="E16" s="21"/>
     </row>
-    <row r="17" spans="2:5" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:5" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B17" s="61"/>
       <c r="C17" s="46" t="s">
         <v>353</v>
@@ -2311,7 +2314,7 @@
       <c r="D17" s="21"/>
       <c r="E17" s="21"/>
     </row>
-    <row r="18" spans="2:5" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:5" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B18" s="60"/>
       <c r="C18" s="46" t="s">
         <v>349</v>
@@ -2319,7 +2322,7 @@
       <c r="D18" s="21"/>
       <c r="E18" s="21"/>
     </row>
-    <row r="19" spans="2:5" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:5" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B19" s="59" t="s">
         <v>337</v>
       </c>
@@ -2329,7 +2332,7 @@
       <c r="D19" s="21"/>
       <c r="E19" s="21"/>
     </row>
-    <row r="20" spans="2:5" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:5" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B20" s="60"/>
       <c r="C20" s="46" t="s">
         <v>348</v>
@@ -2337,7 +2340,7 @@
       <c r="D20" s="21"/>
       <c r="E20" s="21"/>
     </row>
-    <row r="21" spans="2:5" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:5" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B21" s="24" t="s">
         <v>64</v>
       </c>
@@ -2347,7 +2350,7 @@
       <c r="D21" s="21"/>
       <c r="E21" s="21"/>
     </row>
-    <row r="22" spans="2:5" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:5" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B22" s="24" t="s">
         <v>51</v>
       </c>
@@ -2357,7 +2360,7 @@
       <c r="D22" s="21"/>
       <c r="E22" s="21"/>
     </row>
-    <row r="23" spans="2:5" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:5" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B23" s="66" t="s">
         <v>60</v>
       </c>
@@ -2367,7 +2370,7 @@
       <c r="D23" s="21"/>
       <c r="E23" s="21"/>
     </row>
-    <row r="24" spans="2:5" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:5" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B24" s="67"/>
       <c r="C24" s="46" t="s">
         <v>346</v>
@@ -2375,7 +2378,7 @@
       <c r="D24" s="21"/>
       <c r="E24" s="21"/>
     </row>
-    <row r="25" spans="2:5" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:5" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B25" s="24" t="s">
         <v>63</v>
       </c>
@@ -2385,7 +2388,7 @@
       <c r="D25" s="21"/>
       <c r="E25" s="21"/>
     </row>
-    <row r="26" spans="2:5" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:5" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B26" s="24" t="s">
         <v>50</v>
       </c>
@@ -2395,7 +2398,7 @@
       <c r="D26" s="21"/>
       <c r="E26" s="21"/>
     </row>
-    <row r="27" spans="2:5" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:5" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B27" s="24" t="s">
         <v>66</v>
       </c>
@@ -2405,7 +2408,7 @@
       <c r="D27" s="21"/>
       <c r="E27" s="21"/>
     </row>
-    <row r="28" spans="2:5" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:5" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B28" s="24" t="s">
         <v>65</v>
       </c>
@@ -2415,13 +2418,13 @@
       <c r="D28" s="21"/>
       <c r="E28" s="21"/>
     </row>
-    <row r="29" spans="2:5" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:5" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B29" s="23"/>
       <c r="C29" s="21"/>
       <c r="D29" s="21"/>
       <c r="E29" s="21"/>
     </row>
-    <row r="30" spans="2:5" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:5" ht="18" x14ac:dyDescent="0.4">
       <c r="B30" s="19" t="s">
         <v>54</v>
       </c>
@@ -2429,20 +2432,20 @@
       <c r="D30" s="21"/>
       <c r="E30" s="21"/>
     </row>
-    <row r="31" spans="2:5" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:5" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B31" s="21" t="s">
         <v>403</v>
       </c>
       <c r="C31" s="21"/>
       <c r="D31" s="21"/>
     </row>
-    <row r="32" spans="2:5" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:5" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B32" s="21"/>
       <c r="C32" s="21"/>
       <c r="D32" s="21"/>
       <c r="E32" s="21"/>
     </row>
-    <row r="33" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B33" s="49" t="s">
         <v>354</v>
       </c>
@@ -2466,25 +2469,25 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F612F52-003C-4311-BB27-405317FCBADD}">
   <dimension ref="A1:T26"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.08984375" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="1.77734375" style="4" customWidth="1"/>
-    <col min="2" max="2" width="10.44140625" style="4" customWidth="1"/>
+    <col min="1" max="1" width="1.81640625" style="4" customWidth="1"/>
+    <col min="2" max="2" width="10.453125" style="4" customWidth="1"/>
     <col min="3" max="3" width="25" style="4" customWidth="1"/>
-    <col min="4" max="6" width="10.77734375" style="4" customWidth="1"/>
-    <col min="7" max="8" width="10.77734375" style="30" customWidth="1"/>
+    <col min="4" max="6" width="10.81640625" style="4" customWidth="1"/>
+    <col min="7" max="8" width="10.81640625" style="30" customWidth="1"/>
     <col min="9" max="9" width="15" style="30" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.44140625" style="30" customWidth="1"/>
-    <col min="11" max="11" width="12.109375" style="30" bestFit="1" customWidth="1"/>
-    <col min="12" max="15" width="10.77734375" style="30" customWidth="1"/>
-    <col min="16" max="18" width="21.33203125" style="30" customWidth="1"/>
-    <col min="19" max="20" width="9.109375" style="30"/>
-    <col min="21" max="16384" width="9.109375" style="4"/>
+    <col min="10" max="10" width="14.453125" style="30" customWidth="1"/>
+    <col min="11" max="11" width="12.08984375" style="30" bestFit="1" customWidth="1"/>
+    <col min="12" max="15" width="10.81640625" style="30" customWidth="1"/>
+    <col min="16" max="18" width="21.36328125" style="30" customWidth="1"/>
+    <col min="19" max="20" width="9.08984375" style="30"/>
+    <col min="21" max="16384" width="9.08984375" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="69"/>
-      <c r="B1" s="69"/>
+    <row r="1" spans="1:20" ht="12" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="68"/>
+      <c r="B1" s="68"/>
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
@@ -2492,7 +2495,7 @@
       <c r="G1" s="29"/>
       <c r="H1" s="29"/>
     </row>
-    <row r="2" spans="1:20" ht="18" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:20" ht="18.5" x14ac:dyDescent="0.35">
       <c r="A2" s="2"/>
       <c r="B2" s="5" t="s">
         <v>0</v>
@@ -2506,7 +2509,7 @@
       <c r="G2" s="29"/>
       <c r="H2" s="29"/>
     </row>
-    <row r="3" spans="1:20" ht="18" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:20" ht="18.5" x14ac:dyDescent="0.35">
       <c r="A3" s="2"/>
       <c r="B3" s="5" t="s">
         <v>1</v>
@@ -2520,7 +2523,7 @@
       <c r="G3" s="29"/>
       <c r="H3" s="29"/>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A4" s="2"/>
       <c r="B4" s="6" t="s">
         <v>2</v>
@@ -2534,7 +2537,7 @@
       <c r="G4" s="29"/>
       <c r="H4" s="29"/>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A5" s="2"/>
       <c r="B5" s="6" t="s">
         <v>3</v>
@@ -2548,7 +2551,7 @@
       <c r="G5" s="29"/>
       <c r="H5" s="29"/>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A6" s="2"/>
       <c r="B6" s="6" t="s">
         <v>4</v>
@@ -2562,7 +2565,7 @@
       <c r="G6" s="29"/>
       <c r="H6" s="29"/>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="6" t="s">
         <v>6</v>
@@ -2576,7 +2579,7 @@
       <c r="G7" s="29"/>
       <c r="H7" s="29"/>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A8" s="2"/>
       <c r="B8" s="6" t="s">
         <v>7</v>
@@ -2590,7 +2593,7 @@
       <c r="G8" s="29"/>
       <c r="H8" s="29"/>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A9" s="2"/>
       <c r="B9" s="6" t="s">
         <v>9</v>
@@ -2604,9 +2607,9 @@
       <c r="G9" s="29"/>
       <c r="H9" s="29"/>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A10" s="69"/>
-      <c r="B10" s="69"/>
+    <row r="10" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A10" s="68"/>
+      <c r="B10" s="68"/>
       <c r="C10" s="3"/>
       <c r="D10" s="2"/>
       <c r="E10" s="3"/>
@@ -2614,17 +2617,17 @@
       <c r="G10" s="31"/>
       <c r="H10" s="29"/>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A11" s="69"/>
-      <c r="B11" s="69"/>
+    <row r="11" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A11" s="68"/>
+      <c r="B11" s="68"/>
       <c r="C11" s="3"/>
       <c r="D11" s="10"/>
       <c r="E11" s="3"/>
-      <c r="F11" s="68"/>
+      <c r="F11" s="71"/>
       <c r="G11" s="29"/>
       <c r="H11" s="29"/>
     </row>
-    <row r="12" spans="1:20" ht="18" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:20" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A12" s="2"/>
       <c r="B12" s="17" t="s">
         <v>355</v>
@@ -2632,13 +2635,13 @@
       <c r="C12" s="12"/>
       <c r="D12" s="3"/>
       <c r="E12" s="13"/>
-      <c r="F12" s="68"/>
+      <c r="F12" s="71"/>
       <c r="G12" s="29"/>
       <c r="H12" s="29"/>
     </row>
-    <row r="13" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="69"/>
-      <c r="B13" s="69"/>
+    <row r="13" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="68"/>
+      <c r="B13" s="68"/>
       <c r="C13" s="12"/>
       <c r="D13" s="3"/>
       <c r="E13" s="3"/>
@@ -2646,7 +2649,7 @@
       <c r="G13" s="29"/>
       <c r="H13" s="29"/>
     </row>
-    <row r="14" spans="1:20" s="15" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:20" s="15" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A14" s="14"/>
       <c r="B14" s="25" t="s">
         <v>10</v>
@@ -2693,7 +2696,7 @@
       <c r="P14" s="32"/>
       <c r="Q14" s="32"/>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A15" s="3"/>
       <c r="B15" s="43" t="s">
         <v>14</v>
@@ -2742,7 +2745,7 @@
       <c r="S15" s="4"/>
       <c r="T15" s="4"/>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A16" s="3"/>
       <c r="B16" s="1" t="s">
         <v>20</v>
@@ -2791,7 +2794,7 @@
       <c r="S16" s="4"/>
       <c r="T16" s="4"/>
     </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A17" s="3"/>
       <c r="B17" s="1" t="s">
         <v>18</v>
@@ -2840,7 +2843,7 @@
       <c r="S17" s="4"/>
       <c r="T17" s="4"/>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A18" s="3"/>
       <c r="B18" s="1" t="s">
         <v>15</v>
@@ -2889,7 +2892,7 @@
       <c r="S18" s="4"/>
       <c r="T18" s="4"/>
     </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A19" s="3"/>
       <c r="B19" s="1" t="s">
         <v>12</v>
@@ -2938,7 +2941,7 @@
       <c r="S19" s="4"/>
       <c r="T19" s="4"/>
     </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A20" s="3"/>
       <c r="B20" s="1" t="s">
         <v>17</v>
@@ -2987,7 +2990,7 @@
       <c r="S20" s="4"/>
       <c r="T20" s="4"/>
     </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A21" s="3"/>
       <c r="B21" s="1" t="s">
         <v>16</v>
@@ -3036,12 +3039,12 @@
       <c r="S21" s="4"/>
       <c r="T21" s="4"/>
     </row>
-    <row r="22" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A22" s="3"/>
-      <c r="B22" s="70" t="s">
+      <c r="B22" s="69" t="s">
         <v>341</v>
       </c>
-      <c r="C22" s="71"/>
+      <c r="C22" s="70"/>
       <c r="D22" s="45">
         <f t="shared" ref="D22" si="1">SUM(E22:O22)</f>
         <v>10953</v>
@@ -3094,9 +3097,9 @@
       <c r="S22" s="4"/>
       <c r="T22" s="4"/>
     </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A23" s="69"/>
-      <c r="B23" s="69"/>
+    <row r="23" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A23" s="68"/>
+      <c r="B23" s="68"/>
       <c r="C23" s="12"/>
       <c r="D23" s="3"/>
       <c r="E23" s="3"/>
@@ -3104,9 +3107,9 @@
       <c r="G23" s="29"/>
       <c r="H23" s="29"/>
     </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A24" s="69"/>
-      <c r="B24" s="69"/>
+    <row r="24" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A24" s="68"/>
+      <c r="B24" s="68"/>
       <c r="C24" s="12"/>
       <c r="D24" s="3"/>
       <c r="E24" s="3"/>
@@ -3114,9 +3117,9 @@
       <c r="G24" s="29"/>
       <c r="H24" s="29"/>
     </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A25" s="69"/>
-      <c r="B25" s="69"/>
+    <row r="25" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A25" s="68"/>
+      <c r="B25" s="68"/>
       <c r="C25" s="12"/>
       <c r="D25" s="3"/>
       <c r="E25" s="3"/>
@@ -3124,9 +3127,9 @@
       <c r="G25" s="29"/>
       <c r="H25" s="29"/>
     </row>
-    <row r="26" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A26" s="69"/>
-      <c r="B26" s="69"/>
+    <row r="26" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A26" s="68"/>
+      <c r="B26" s="68"/>
       <c r="C26" s="12"/>
       <c r="D26" s="3"/>
       <c r="E26" s="3"/>
@@ -3149,16 +3152,16 @@
     <sortCondition ref="B15:B21"/>
   </sortState>
   <mergeCells count="10">
+    <mergeCell ref="F11:F12"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="A11:B11"/>
     <mergeCell ref="A24:B24"/>
     <mergeCell ref="A25:B25"/>
     <mergeCell ref="A26:B26"/>
     <mergeCell ref="B22:C22"/>
     <mergeCell ref="A23:B23"/>
-    <mergeCell ref="F11:F12"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="A11:B11"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C9" r:id="rId1" xr:uid="{424343C5-7BA4-4062-84AD-C2B156F05DFF}"/>
@@ -3171,29 +3174,29 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54853DFE-3DA2-4431-9118-18B40B4CEBE8}">
   <dimension ref="A1:V151"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.08984375" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="1.44140625" style="4" customWidth="1"/>
+    <col min="1" max="1" width="1.453125" style="4" customWidth="1"/>
     <col min="2" max="2" width="11" style="4" customWidth="1"/>
     <col min="3" max="3" width="25" style="4" customWidth="1"/>
-    <col min="4" max="4" width="57.5546875" style="4" customWidth="1"/>
-    <col min="5" max="5" width="29.88671875" style="4" customWidth="1"/>
-    <col min="6" max="6" width="12.21875" style="4" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="71.109375" style="4" customWidth="1"/>
-    <col min="8" max="8" width="10.6640625" style="4" customWidth="1"/>
-    <col min="9" max="12" width="10.6640625" style="30" customWidth="1"/>
+    <col min="4" max="4" width="57.54296875" style="4" customWidth="1"/>
+    <col min="5" max="5" width="29.90625" style="4" customWidth="1"/>
+    <col min="6" max="6" width="12.1796875" style="4" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="71.08984375" style="4" customWidth="1"/>
+    <col min="8" max="8" width="10.6328125" style="4" customWidth="1"/>
+    <col min="9" max="12" width="10.6328125" style="30" customWidth="1"/>
     <col min="13" max="13" width="15" style="30" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="14.109375" style="30" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.109375" style="30" bestFit="1" customWidth="1"/>
-    <col min="16" max="19" width="10.6640625" style="30" customWidth="1"/>
-    <col min="20" max="20" width="21.33203125" style="30" customWidth="1"/>
-    <col min="21" max="22" width="9.109375" style="30"/>
-    <col min="23" max="16384" width="9.109375" style="4"/>
+    <col min="14" max="14" width="14.08984375" style="30" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.08984375" style="30" bestFit="1" customWidth="1"/>
+    <col min="16" max="19" width="10.6328125" style="30" customWidth="1"/>
+    <col min="20" max="20" width="21.36328125" style="30" customWidth="1"/>
+    <col min="21" max="22" width="9.08984375" style="30"/>
+    <col min="23" max="16384" width="9.08984375" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" ht="9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="69"/>
-      <c r="B1" s="69"/>
+    <row r="1" spans="1:22" ht="9" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="68"/>
+      <c r="B1" s="68"/>
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
@@ -3203,7 +3206,7 @@
       <c r="I1" s="29"/>
       <c r="J1" s="29"/>
     </row>
-    <row r="2" spans="1:22" ht="18" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:22" ht="18.5" x14ac:dyDescent="0.35">
       <c r="A2" s="2"/>
       <c r="B2" s="5" t="s">
         <v>0</v>
@@ -3219,7 +3222,7 @@
       <c r="I2" s="29"/>
       <c r="J2" s="29"/>
     </row>
-    <row r="3" spans="1:22" ht="18" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:22" ht="18.5" x14ac:dyDescent="0.35">
       <c r="A3" s="2"/>
       <c r="B3" s="5" t="s">
         <v>1</v>
@@ -3235,7 +3238,7 @@
       <c r="I3" s="29"/>
       <c r="J3" s="29"/>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A4" s="2"/>
       <c r="B4" s="6" t="s">
         <v>2</v>
@@ -3251,7 +3254,7 @@
       <c r="I4" s="29"/>
       <c r="J4" s="29"/>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A5" s="2"/>
       <c r="B5" s="6" t="s">
         <v>3</v>
@@ -3267,7 +3270,7 @@
       <c r="I5" s="29"/>
       <c r="J5" s="29"/>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A6" s="2"/>
       <c r="B6" s="6" t="s">
         <v>4</v>
@@ -3283,7 +3286,7 @@
       <c r="I6" s="29"/>
       <c r="J6" s="29"/>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="6" t="s">
         <v>6</v>
@@ -3299,7 +3302,7 @@
       <c r="I7" s="29"/>
       <c r="J7" s="29"/>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A8" s="2"/>
       <c r="B8" s="6" t="s">
         <v>7</v>
@@ -3315,7 +3318,7 @@
       <c r="I8" s="29"/>
       <c r="J8" s="29"/>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A9" s="2"/>
       <c r="B9" s="6" t="s">
         <v>9</v>
@@ -3331,9 +3334,9 @@
       <c r="I9" s="29"/>
       <c r="J9" s="29"/>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A10" s="69"/>
-      <c r="B10" s="69"/>
+    <row r="10" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A10" s="68"/>
+      <c r="B10" s="68"/>
       <c r="C10" s="3"/>
       <c r="D10" s="3"/>
       <c r="E10" s="3"/>
@@ -3343,19 +3346,19 @@
       <c r="I10" s="29"/>
       <c r="J10" s="29"/>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A11" s="69"/>
-      <c r="B11" s="69"/>
+    <row r="11" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A11" s="68"/>
+      <c r="B11" s="68"/>
       <c r="C11" s="3"/>
       <c r="D11" s="3"/>
       <c r="E11" s="10"/>
       <c r="F11" s="10"/>
       <c r="G11" s="3"/>
-      <c r="H11" s="68"/>
+      <c r="H11" s="71"/>
       <c r="I11" s="29"/>
       <c r="J11" s="29"/>
     </row>
-    <row r="12" spans="1:22" ht="18" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:22" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A12" s="2"/>
       <c r="B12" s="17" t="s">
         <v>356</v>
@@ -3365,13 +3368,13 @@
       <c r="E12" s="3"/>
       <c r="F12" s="3"/>
       <c r="G12" s="13"/>
-      <c r="H12" s="68"/>
+      <c r="H12" s="71"/>
       <c r="I12" s="29"/>
       <c r="J12" s="29"/>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A13" s="69"/>
-      <c r="B13" s="69"/>
+    <row r="13" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A13" s="68"/>
+      <c r="B13" s="68"/>
       <c r="C13" s="12"/>
       <c r="D13" s="3"/>
       <c r="E13" s="3"/>
@@ -3391,7 +3394,7 @@
       <c r="S13" s="29"/>
       <c r="T13" s="29"/>
     </row>
-    <row r="14" spans="1:22" s="39" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:22" s="39" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="48"/>
       <c r="B14" s="25" t="s">
         <v>10</v>
@@ -3450,7 +3453,7 @@
       <c r="T14" s="38"/>
       <c r="U14" s="38"/>
     </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A15" s="2"/>
       <c r="B15" s="1" t="s">
         <v>14</v>
@@ -3509,7 +3512,7 @@
       </c>
       <c r="V15" s="4"/>
     </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A16" s="2"/>
       <c r="B16" s="1" t="s">
         <v>14</v>
@@ -3568,7 +3571,7 @@
       </c>
       <c r="V16" s="4"/>
     </row>
-    <row r="17" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A17" s="2"/>
       <c r="B17" s="1" t="s">
         <v>14</v>
@@ -3627,7 +3630,7 @@
       </c>
       <c r="V17" s="4"/>
     </row>
-    <row r="18" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A18" s="2"/>
       <c r="B18" s="1" t="s">
         <v>14</v>
@@ -3686,7 +3689,7 @@
       </c>
       <c r="V18" s="4"/>
     </row>
-    <row r="19" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A19" s="2"/>
       <c r="B19" s="1" t="s">
         <v>14</v>
@@ -3745,7 +3748,7 @@
       </c>
       <c r="V19" s="4"/>
     </row>
-    <row r="20" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A20" s="2"/>
       <c r="B20" s="1" t="s">
         <v>14</v>
@@ -3804,7 +3807,7 @@
       </c>
       <c r="V20" s="4"/>
     </row>
-    <row r="21" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A21" s="2"/>
       <c r="B21" s="1" t="s">
         <v>14</v>
@@ -3863,7 +3866,7 @@
       </c>
       <c r="V21" s="4"/>
     </row>
-    <row r="22" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A22" s="2"/>
       <c r="B22" s="1" t="s">
         <v>14</v>
@@ -3922,7 +3925,7 @@
       </c>
       <c r="V22" s="4"/>
     </row>
-    <row r="23" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A23" s="2"/>
       <c r="B23" s="1" t="s">
         <v>14</v>
@@ -3981,7 +3984,7 @@
       </c>
       <c r="V23" s="4"/>
     </row>
-    <row r="24" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A24" s="2"/>
       <c r="B24" s="1" t="s">
         <v>14</v>
@@ -4040,7 +4043,7 @@
       </c>
       <c r="V24" s="4"/>
     </row>
-    <row r="25" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A25" s="2"/>
       <c r="B25" s="1" t="s">
         <v>14</v>
@@ -4099,7 +4102,7 @@
       </c>
       <c r="V25" s="4"/>
     </row>
-    <row r="26" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A26" s="2"/>
       <c r="B26" s="1" t="s">
         <v>14</v>
@@ -4158,7 +4161,7 @@
       </c>
       <c r="V26" s="4"/>
     </row>
-    <row r="27" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A27" s="2"/>
       <c r="B27" s="1" t="s">
         <v>14</v>
@@ -4217,7 +4220,7 @@
       </c>
       <c r="V27" s="4"/>
     </row>
-    <row r="28" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A28" s="2"/>
       <c r="B28" s="1" t="s">
         <v>14</v>
@@ -4276,7 +4279,7 @@
       </c>
       <c r="V28" s="4"/>
     </row>
-    <row r="29" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A29" s="2"/>
       <c r="B29" s="1" t="s">
         <v>14</v>
@@ -4335,7 +4338,7 @@
       </c>
       <c r="V29" s="4"/>
     </row>
-    <row r="30" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A30" s="2"/>
       <c r="B30" s="1" t="s">
         <v>14</v>
@@ -4394,7 +4397,7 @@
       </c>
       <c r="V30" s="4"/>
     </row>
-    <row r="31" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A31" s="2"/>
       <c r="B31" s="1" t="s">
         <v>14</v>
@@ -4453,7 +4456,7 @@
       </c>
       <c r="V31" s="4"/>
     </row>
-    <row r="32" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A32" s="2"/>
       <c r="B32" s="1" t="s">
         <v>14</v>
@@ -4512,7 +4515,7 @@
       </c>
       <c r="V32" s="4"/>
     </row>
-    <row r="33" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A33" s="2"/>
       <c r="B33" s="1" t="s">
         <v>14</v>
@@ -4571,7 +4574,7 @@
       </c>
       <c r="V33" s="4"/>
     </row>
-    <row r="34" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A34" s="2"/>
       <c r="B34" s="1" t="s">
         <v>14</v>
@@ -4630,7 +4633,7 @@
       </c>
       <c r="V34" s="4"/>
     </row>
-    <row r="35" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A35" s="2"/>
       <c r="B35" s="1" t="s">
         <v>14</v>
@@ -4689,7 +4692,7 @@
       </c>
       <c r="V35" s="4"/>
     </row>
-    <row r="36" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A36" s="2"/>
       <c r="B36" s="1" t="s">
         <v>14</v>
@@ -4748,7 +4751,7 @@
       </c>
       <c r="V36" s="4"/>
     </row>
-    <row r="37" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A37" s="2"/>
       <c r="B37" s="1" t="s">
         <v>20</v>
@@ -4807,7 +4810,7 @@
       </c>
       <c r="V37" s="4"/>
     </row>
-    <row r="38" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A38" s="2"/>
       <c r="B38" s="1" t="s">
         <v>20</v>
@@ -4866,7 +4869,7 @@
       </c>
       <c r="V38" s="4"/>
     </row>
-    <row r="39" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A39" s="2"/>
       <c r="B39" s="1" t="s">
         <v>20</v>
@@ -4925,7 +4928,7 @@
       </c>
       <c r="V39" s="4"/>
     </row>
-    <row r="40" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A40" s="2"/>
       <c r="B40" s="1" t="s">
         <v>20</v>
@@ -4984,7 +4987,7 @@
       </c>
       <c r="V40" s="4"/>
     </row>
-    <row r="41" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A41" s="2"/>
       <c r="B41" s="1" t="s">
         <v>20</v>
@@ -5043,7 +5046,7 @@
       </c>
       <c r="V41" s="4"/>
     </row>
-    <row r="42" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A42" s="2"/>
       <c r="B42" s="1" t="s">
         <v>20</v>
@@ -5102,7 +5105,7 @@
       </c>
       <c r="V42" s="4"/>
     </row>
-    <row r="43" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A43" s="2"/>
       <c r="B43" s="1" t="s">
         <v>20</v>
@@ -5161,7 +5164,7 @@
       </c>
       <c r="V43" s="4"/>
     </row>
-    <row r="44" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A44" s="2"/>
       <c r="B44" s="1" t="s">
         <v>20</v>
@@ -5220,7 +5223,7 @@
       </c>
       <c r="V44" s="4"/>
     </row>
-    <row r="45" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A45" s="2"/>
       <c r="B45" s="1" t="s">
         <v>20</v>
@@ -5279,7 +5282,7 @@
       </c>
       <c r="V45" s="4"/>
     </row>
-    <row r="46" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A46" s="2"/>
       <c r="B46" s="1" t="s">
         <v>20</v>
@@ -5338,7 +5341,7 @@
       </c>
       <c r="V46" s="4"/>
     </row>
-    <row r="47" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A47" s="2"/>
       <c r="B47" s="1" t="s">
         <v>20</v>
@@ -5397,7 +5400,7 @@
       </c>
       <c r="V47" s="4"/>
     </row>
-    <row r="48" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A48" s="2"/>
       <c r="B48" s="1" t="s">
         <v>20</v>
@@ -5456,7 +5459,7 @@
       </c>
       <c r="V48" s="4"/>
     </row>
-    <row r="49" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A49" s="2"/>
       <c r="B49" s="1" t="s">
         <v>20</v>
@@ -5515,7 +5518,7 @@
       </c>
       <c r="V49" s="4"/>
     </row>
-    <row r="50" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B50" s="1" t="s">
         <v>20</v>
       </c>
@@ -5573,7 +5576,7 @@
       </c>
       <c r="V50" s="4"/>
     </row>
-    <row r="51" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B51" s="1" t="s">
         <v>18</v>
       </c>
@@ -5631,7 +5634,7 @@
       </c>
       <c r="V51" s="4"/>
     </row>
-    <row r="52" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B52" s="1" t="s">
         <v>18</v>
       </c>
@@ -5689,7 +5692,7 @@
       </c>
       <c r="V52" s="4"/>
     </row>
-    <row r="53" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B53" s="1" t="s">
         <v>18</v>
       </c>
@@ -5747,7 +5750,7 @@
       </c>
       <c r="V53" s="4"/>
     </row>
-    <row r="54" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B54" s="1" t="s">
         <v>18</v>
       </c>
@@ -5805,7 +5808,7 @@
       </c>
       <c r="V54" s="4"/>
     </row>
-    <row r="55" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B55" s="1" t="s">
         <v>18</v>
       </c>
@@ -5863,7 +5866,7 @@
       </c>
       <c r="V55" s="4"/>
     </row>
-    <row r="56" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B56" s="1" t="s">
         <v>18</v>
       </c>
@@ -5921,7 +5924,7 @@
       </c>
       <c r="V56" s="4"/>
     </row>
-    <row r="57" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B57" s="1" t="s">
         <v>18</v>
       </c>
@@ -5979,7 +5982,7 @@
       </c>
       <c r="V57" s="4"/>
     </row>
-    <row r="58" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B58" s="1" t="s">
         <v>18</v>
       </c>
@@ -6037,7 +6040,7 @@
       </c>
       <c r="V58" s="4"/>
     </row>
-    <row r="59" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B59" s="1" t="s">
         <v>18</v>
       </c>
@@ -6095,7 +6098,7 @@
       </c>
       <c r="V59" s="4"/>
     </row>
-    <row r="60" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B60" s="1" t="s">
         <v>18</v>
       </c>
@@ -6153,7 +6156,7 @@
       </c>
       <c r="V60" s="4"/>
     </row>
-    <row r="61" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B61" s="1" t="s">
         <v>18</v>
       </c>
@@ -6211,7 +6214,7 @@
       </c>
       <c r="V61" s="4"/>
     </row>
-    <row r="62" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B62" s="1" t="s">
         <v>18</v>
       </c>
@@ -6269,7 +6272,7 @@
       </c>
       <c r="V62" s="4"/>
     </row>
-    <row r="63" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B63" s="1" t="s">
         <v>18</v>
       </c>
@@ -6327,7 +6330,7 @@
       </c>
       <c r="V63" s="4"/>
     </row>
-    <row r="64" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:22" x14ac:dyDescent="0.35">
       <c r="B64" s="1" t="s">
         <v>18</v>
       </c>
@@ -6385,7 +6388,7 @@
       </c>
       <c r="V64" s="4"/>
     </row>
-    <row r="65" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="65" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B65" s="1" t="s">
         <v>18</v>
       </c>
@@ -6443,7 +6446,7 @@
       </c>
       <c r="V65" s="4"/>
     </row>
-    <row r="66" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="66" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B66" s="1" t="s">
         <v>18</v>
       </c>
@@ -6501,7 +6504,7 @@
       </c>
       <c r="V66" s="4"/>
     </row>
-    <row r="67" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="67" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B67" s="1" t="s">
         <v>18</v>
       </c>
@@ -6559,7 +6562,7 @@
       </c>
       <c r="V67" s="4"/>
     </row>
-    <row r="68" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="68" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B68" s="1" t="s">
         <v>18</v>
       </c>
@@ -6617,7 +6620,7 @@
       </c>
       <c r="V68" s="4"/>
     </row>
-    <row r="69" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="69" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B69" s="1" t="s">
         <v>15</v>
       </c>
@@ -6675,7 +6678,7 @@
       </c>
       <c r="V69" s="4"/>
     </row>
-    <row r="70" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="70" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B70" s="1" t="s">
         <v>15</v>
       </c>
@@ -6733,7 +6736,7 @@
       </c>
       <c r="V70" s="4"/>
     </row>
-    <row r="71" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="71" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B71" s="1" t="s">
         <v>15</v>
       </c>
@@ -6791,7 +6794,7 @@
       </c>
       <c r="V71" s="4"/>
     </row>
-    <row r="72" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="72" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B72" s="1" t="s">
         <v>15</v>
       </c>
@@ -6849,7 +6852,7 @@
       </c>
       <c r="V72" s="4"/>
     </row>
-    <row r="73" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="73" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B73" s="1" t="s">
         <v>15</v>
       </c>
@@ -6907,7 +6910,7 @@
       </c>
       <c r="V73" s="4"/>
     </row>
-    <row r="74" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="74" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B74" s="1" t="s">
         <v>15</v>
       </c>
@@ -6965,7 +6968,7 @@
       </c>
       <c r="V74" s="4"/>
     </row>
-    <row r="75" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="75" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B75" s="1" t="s">
         <v>15</v>
       </c>
@@ -7023,7 +7026,7 @@
       </c>
       <c r="V75" s="4"/>
     </row>
-    <row r="76" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="76" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B76" s="1" t="s">
         <v>15</v>
       </c>
@@ -7081,7 +7084,7 @@
       </c>
       <c r="V76" s="4"/>
     </row>
-    <row r="77" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="77" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B77" s="1" t="s">
         <v>15</v>
       </c>
@@ -7139,7 +7142,7 @@
       </c>
       <c r="V77" s="4"/>
     </row>
-    <row r="78" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="78" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B78" s="1" t="s">
         <v>15</v>
       </c>
@@ -7197,7 +7200,7 @@
       </c>
       <c r="V78" s="4"/>
     </row>
-    <row r="79" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="79" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B79" s="1" t="s">
         <v>15</v>
       </c>
@@ -7255,7 +7258,7 @@
       </c>
       <c r="V79" s="4"/>
     </row>
-    <row r="80" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="80" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B80" s="1" t="s">
         <v>15</v>
       </c>
@@ -7313,7 +7316,7 @@
       </c>
       <c r="V80" s="4"/>
     </row>
-    <row r="81" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="81" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B81" s="1" t="s">
         <v>15</v>
       </c>
@@ -7371,7 +7374,7 @@
       </c>
       <c r="V81" s="4"/>
     </row>
-    <row r="82" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="82" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B82" s="1" t="s">
         <v>15</v>
       </c>
@@ -7429,7 +7432,7 @@
       </c>
       <c r="V82" s="4"/>
     </row>
-    <row r="83" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="83" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B83" s="1" t="s">
         <v>15</v>
       </c>
@@ -7487,7 +7490,7 @@
       </c>
       <c r="V83" s="4"/>
     </row>
-    <row r="84" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="84" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B84" s="1" t="s">
         <v>15</v>
       </c>
@@ -7545,7 +7548,7 @@
       </c>
       <c r="V84" s="4"/>
     </row>
-    <row r="85" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="85" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B85" s="1" t="s">
         <v>15</v>
       </c>
@@ -7603,7 +7606,7 @@
       </c>
       <c r="V85" s="4"/>
     </row>
-    <row r="86" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="86" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B86" s="1" t="s">
         <v>15</v>
       </c>
@@ -7661,7 +7664,7 @@
       </c>
       <c r="V86" s="4"/>
     </row>
-    <row r="87" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="87" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B87" s="1" t="s">
         <v>15</v>
       </c>
@@ -7719,7 +7722,7 @@
       </c>
       <c r="V87" s="4"/>
     </row>
-    <row r="88" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="88" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B88" s="1" t="s">
         <v>15</v>
       </c>
@@ -7777,7 +7780,7 @@
       </c>
       <c r="V88" s="4"/>
     </row>
-    <row r="89" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="89" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B89" s="1" t="s">
         <v>15</v>
       </c>
@@ -7835,7 +7838,7 @@
       </c>
       <c r="V89" s="4"/>
     </row>
-    <row r="90" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="90" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B90" s="1" t="s">
         <v>15</v>
       </c>
@@ -7893,7 +7896,7 @@
       </c>
       <c r="V90" s="4"/>
     </row>
-    <row r="91" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="91" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B91" s="1" t="s">
         <v>15</v>
       </c>
@@ -7951,7 +7954,7 @@
       </c>
       <c r="V91" s="4"/>
     </row>
-    <row r="92" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="92" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B92" s="1" t="s">
         <v>12</v>
       </c>
@@ -8009,7 +8012,7 @@
       </c>
       <c r="V92" s="4"/>
     </row>
-    <row r="93" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="93" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B93" s="1" t="s">
         <v>12</v>
       </c>
@@ -8067,7 +8070,7 @@
       </c>
       <c r="V93" s="4"/>
     </row>
-    <row r="94" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="94" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B94" s="1" t="s">
         <v>12</v>
       </c>
@@ -8125,7 +8128,7 @@
       </c>
       <c r="V94" s="4"/>
     </row>
-    <row r="95" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="95" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B95" s="1" t="s">
         <v>12</v>
       </c>
@@ -8183,7 +8186,7 @@
       </c>
       <c r="V95" s="4"/>
     </row>
-    <row r="96" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="96" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B96" s="1" t="s">
         <v>12</v>
       </c>
@@ -8241,7 +8244,7 @@
       </c>
       <c r="V96" s="4"/>
     </row>
-    <row r="97" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="97" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B97" s="1" t="s">
         <v>12</v>
       </c>
@@ -8299,7 +8302,7 @@
       </c>
       <c r="V97" s="4"/>
     </row>
-    <row r="98" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="98" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B98" s="1" t="s">
         <v>12</v>
       </c>
@@ -8357,7 +8360,7 @@
       </c>
       <c r="V98" s="4"/>
     </row>
-    <row r="99" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="99" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B99" s="1" t="s">
         <v>12</v>
       </c>
@@ -8415,7 +8418,7 @@
       </c>
       <c r="V99" s="4"/>
     </row>
-    <row r="100" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="100" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B100" s="1" t="s">
         <v>12</v>
       </c>
@@ -8473,7 +8476,7 @@
       </c>
       <c r="V100" s="4"/>
     </row>
-    <row r="101" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="101" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B101" s="1" t="s">
         <v>12</v>
       </c>
@@ -8531,7 +8534,7 @@
       </c>
       <c r="V101" s="4"/>
     </row>
-    <row r="102" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="102" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B102" s="1" t="s">
         <v>12</v>
       </c>
@@ -8589,7 +8592,7 @@
       </c>
       <c r="V102" s="4"/>
     </row>
-    <row r="103" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="103" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B103" s="1" t="s">
         <v>12</v>
       </c>
@@ -8647,7 +8650,7 @@
       </c>
       <c r="V103" s="4"/>
     </row>
-    <row r="104" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="104" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B104" s="1" t="s">
         <v>12</v>
       </c>
@@ -8705,7 +8708,7 @@
       </c>
       <c r="V104" s="4"/>
     </row>
-    <row r="105" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="105" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B105" s="1" t="s">
         <v>12</v>
       </c>
@@ -8763,7 +8766,7 @@
       </c>
       <c r="V105" s="4"/>
     </row>
-    <row r="106" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="106" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B106" s="1" t="s">
         <v>17</v>
       </c>
@@ -8821,7 +8824,7 @@
       </c>
       <c r="V106" s="4"/>
     </row>
-    <row r="107" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="107" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B107" s="1" t="s">
         <v>17</v>
       </c>
@@ -8879,7 +8882,7 @@
       </c>
       <c r="V107" s="4"/>
     </row>
-    <row r="108" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="108" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B108" s="1" t="s">
         <v>17</v>
       </c>
@@ -8937,7 +8940,7 @@
       </c>
       <c r="V108" s="4"/>
     </row>
-    <row r="109" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="109" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B109" s="1" t="s">
         <v>17</v>
       </c>
@@ -8995,7 +8998,7 @@
       </c>
       <c r="V109" s="4"/>
     </row>
-    <row r="110" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="110" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B110" s="1" t="s">
         <v>17</v>
       </c>
@@ -9053,7 +9056,7 @@
       </c>
       <c r="V110" s="4"/>
     </row>
-    <row r="111" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="111" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B111" s="1" t="s">
         <v>17</v>
       </c>
@@ -9111,7 +9114,7 @@
       </c>
       <c r="V111" s="4"/>
     </row>
-    <row r="112" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="112" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B112" s="1" t="s">
         <v>17</v>
       </c>
@@ -9169,7 +9172,7 @@
       </c>
       <c r="V112" s="4"/>
     </row>
-    <row r="113" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="113" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B113" s="1" t="s">
         <v>17</v>
       </c>
@@ -9227,7 +9230,7 @@
       </c>
       <c r="V113" s="4"/>
     </row>
-    <row r="114" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="114" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B114" s="1" t="s">
         <v>17</v>
       </c>
@@ -9285,7 +9288,7 @@
       </c>
       <c r="V114" s="4"/>
     </row>
-    <row r="115" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="115" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B115" s="1" t="s">
         <v>17</v>
       </c>
@@ -9343,7 +9346,7 @@
       </c>
       <c r="V115" s="4"/>
     </row>
-    <row r="116" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="116" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B116" s="1" t="s">
         <v>17</v>
       </c>
@@ -9401,7 +9404,7 @@
       </c>
       <c r="V116" s="4"/>
     </row>
-    <row r="117" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="117" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B117" s="1" t="s">
         <v>17</v>
       </c>
@@ -9459,7 +9462,7 @@
       </c>
       <c r="V117" s="4"/>
     </row>
-    <row r="118" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="118" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B118" s="1" t="s">
         <v>17</v>
       </c>
@@ -9517,7 +9520,7 @@
       </c>
       <c r="V118" s="4"/>
     </row>
-    <row r="119" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="119" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B119" s="1" t="s">
         <v>17</v>
       </c>
@@ -9575,7 +9578,7 @@
       </c>
       <c r="V119" s="4"/>
     </row>
-    <row r="120" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="120" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B120" s="1" t="s">
         <v>17</v>
       </c>
@@ -9633,7 +9636,7 @@
       </c>
       <c r="V120" s="4"/>
     </row>
-    <row r="121" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="121" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B121" s="1" t="s">
         <v>17</v>
       </c>
@@ -9691,7 +9694,7 @@
       </c>
       <c r="V121" s="4"/>
     </row>
-    <row r="122" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="122" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B122" s="1" t="s">
         <v>17</v>
       </c>
@@ -9749,7 +9752,7 @@
       </c>
       <c r="V122" s="4"/>
     </row>
-    <row r="123" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="123" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B123" s="1" t="s">
         <v>17</v>
       </c>
@@ -9807,7 +9810,7 @@
       </c>
       <c r="V123" s="4"/>
     </row>
-    <row r="124" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="124" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B124" s="1" t="s">
         <v>17</v>
       </c>
@@ -9865,7 +9868,7 @@
       </c>
       <c r="V124" s="4"/>
     </row>
-    <row r="125" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="125" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B125" s="1" t="s">
         <v>17</v>
       </c>
@@ -9923,7 +9926,7 @@
       </c>
       <c r="V125" s="4"/>
     </row>
-    <row r="126" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="126" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B126" s="1" t="s">
         <v>17</v>
       </c>
@@ -9981,7 +9984,7 @@
       </c>
       <c r="V126" s="4"/>
     </row>
-    <row r="127" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="127" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B127" s="1" t="s">
         <v>17</v>
       </c>
@@ -10039,7 +10042,7 @@
       </c>
       <c r="V127" s="4"/>
     </row>
-    <row r="128" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="128" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B128" s="1" t="s">
         <v>17</v>
       </c>
@@ -10097,7 +10100,7 @@
       </c>
       <c r="V128" s="4"/>
     </row>
-    <row r="129" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="129" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B129" s="1" t="s">
         <v>17</v>
       </c>
@@ -10155,7 +10158,7 @@
       </c>
       <c r="V129" s="4"/>
     </row>
-    <row r="130" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="130" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B130" s="1" t="s">
         <v>16</v>
       </c>
@@ -10213,7 +10216,7 @@
       </c>
       <c r="V130" s="4"/>
     </row>
-    <row r="131" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="131" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B131" s="1" t="s">
         <v>16</v>
       </c>
@@ -10271,7 +10274,7 @@
       </c>
       <c r="V131" s="4"/>
     </row>
-    <row r="132" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="132" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B132" s="1" t="s">
         <v>16</v>
       </c>
@@ -10329,7 +10332,7 @@
       </c>
       <c r="V132" s="4"/>
     </row>
-    <row r="133" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="133" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B133" s="1" t="s">
         <v>16</v>
       </c>
@@ -10387,7 +10390,7 @@
       </c>
       <c r="V133" s="4"/>
     </row>
-    <row r="134" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="134" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B134" s="1" t="s">
         <v>16</v>
       </c>
@@ -10445,7 +10448,7 @@
       </c>
       <c r="V134" s="4"/>
     </row>
-    <row r="135" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="135" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B135" s="1" t="s">
         <v>16</v>
       </c>
@@ -10503,7 +10506,7 @@
       </c>
       <c r="V135" s="4"/>
     </row>
-    <row r="136" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="136" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B136" s="1" t="s">
         <v>16</v>
       </c>
@@ -10561,7 +10564,7 @@
       </c>
       <c r="V136" s="4"/>
     </row>
-    <row r="137" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="137" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B137" s="1" t="s">
         <v>16</v>
       </c>
@@ -10619,7 +10622,7 @@
       </c>
       <c r="V137" s="4"/>
     </row>
-    <row r="138" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="138" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B138" s="1" t="s">
         <v>16</v>
       </c>
@@ -10677,7 +10680,7 @@
       </c>
       <c r="V138" s="4"/>
     </row>
-    <row r="139" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="139" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B139" s="1" t="s">
         <v>16</v>
       </c>
@@ -10735,7 +10738,7 @@
       </c>
       <c r="V139" s="4"/>
     </row>
-    <row r="140" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="140" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B140" s="1" t="s">
         <v>16</v>
       </c>
@@ -10793,7 +10796,7 @@
       </c>
       <c r="V140" s="4"/>
     </row>
-    <row r="141" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="141" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B141" s="1" t="s">
         <v>16</v>
       </c>
@@ -10851,7 +10854,7 @@
       </c>
       <c r="V141" s="4"/>
     </row>
-    <row r="142" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="142" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B142" s="1" t="s">
         <v>16</v>
       </c>
@@ -10909,7 +10912,7 @@
       </c>
       <c r="V142" s="4"/>
     </row>
-    <row r="143" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="143" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B143" s="1" t="s">
         <v>16</v>
       </c>
@@ -10929,7 +10932,7 @@
         <v>216</v>
       </c>
       <c r="H143" s="45">
-        <f t="shared" ref="H143:H174" si="4">SUM(I143:S143)</f>
+        <f t="shared" ref="H143:H151" si="4">SUM(I143:S143)</f>
         <v>22</v>
       </c>
       <c r="I143" s="34">
@@ -10967,7 +10970,7 @@
       </c>
       <c r="V143" s="4"/>
     </row>
-    <row r="144" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="144" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B144" s="1" t="s">
         <v>16</v>
       </c>
@@ -11025,7 +11028,7 @@
       </c>
       <c r="V144" s="4"/>
     </row>
-    <row r="145" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="145" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B145" s="1" t="s">
         <v>16</v>
       </c>
@@ -11083,7 +11086,7 @@
       </c>
       <c r="V145" s="4"/>
     </row>
-    <row r="146" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="146" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B146" s="1" t="s">
         <v>16</v>
       </c>
@@ -11141,7 +11144,7 @@
       </c>
       <c r="V146" s="4"/>
     </row>
-    <row r="147" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="147" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B147" s="1" t="s">
         <v>16</v>
       </c>
@@ -11199,7 +11202,7 @@
       </c>
       <c r="V147" s="4"/>
     </row>
-    <row r="148" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="148" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B148" s="1" t="s">
         <v>16</v>
       </c>
@@ -11257,7 +11260,7 @@
       </c>
       <c r="V148" s="4"/>
     </row>
-    <row r="149" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="149" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B149" s="1" t="s">
         <v>16</v>
       </c>
@@ -11315,7 +11318,7 @@
       </c>
       <c r="V149" s="4"/>
     </row>
-    <row r="150" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="150" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B150" s="1" t="s">
         <v>16</v>
       </c>
@@ -11373,7 +11376,7 @@
       </c>
       <c r="V150" s="4"/>
     </row>
-    <row r="151" spans="2:22" x14ac:dyDescent="0.3">
+    <row r="151" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B151" s="1" t="s">
         <v>16</v>
       </c>
@@ -11432,6 +11435,7 @@
       <c r="V151" s="4"/>
     </row>
   </sheetData>
+  <autoFilter ref="A14:V151" xr:uid="{54853DFE-3DA2-4431-9118-18B40B4CEBE8}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B15:S151">
     <sortCondition ref="B15:B151"/>
     <sortCondition ref="E15:E151"/>
@@ -11454,6 +11458,36 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <Person xmlns="7ac25642-bc50-40b5-aee4-3aad54522c8e">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Person>
+    <Review_x0020_Date xmlns="7ac25642-bc50-40b5-aee4-3aad54522c8e" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7ac25642-bc50-40b5-aee4-3aad54522c8e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="cccaf3ac-2de9-44d4-aa31-54302fceb5f7" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101007B3BB9CF23C28F40815860AD19EBF8D8" ma:contentTypeVersion="69" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="c27dc56a182141f0a236d562ca3d8131">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="22284d95-5a94-4052-8e65-be8da71d5f72" xmlns:ns3="7ac25642-bc50-40b5-aee4-3aad54522c8e" xmlns:ns4="51bfcd92-eb3e-40f4-8778-2bbfb88a890b" xmlns:ns5="cccaf3ac-2de9-44d4-aa31-54302fceb5f7" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="404f797f4b8bf9f41e2eaefa8a1e7b93" ns1:_="" ns2:_="" ns3:_="" ns4:_="" ns5:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -11719,37 +11753,35 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7706BC6D-3A42-4EE7-8F02-E43240B61A4E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="7ac25642-bc50-40b5-aee4-3aad54522c8e"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="22284d95-5a94-4052-8e65-be8da71d5f72"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="51bfcd92-eb3e-40f4-8778-2bbfb88a890b"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="cccaf3ac-2de9-44d4-aa31-54302fceb5f7"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <Person xmlns="7ac25642-bc50-40b5-aee4-3aad54522c8e">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </Person>
-    <Review_x0020_Date xmlns="7ac25642-bc50-40b5-aee4-3aad54522c8e" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7ac25642-bc50-40b5-aee4-3aad54522c8e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="cccaf3ac-2de9-44d4-aa31-54302fceb5f7" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F436471D-C45C-4DAE-8C21-752C3CF7A405}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7125CEC8-7CEB-4E5D-9AA9-68B2907216A9}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -11769,32 +11801,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F436471D-C45C-4DAE-8C21-752C3CF7A405}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7706BC6D-3A42-4EE7-8F02-E43240B61A4E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="7ac25642-bc50-40b5-aee4-3aad54522c8e"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="22284d95-5a94-4052-8e65-be8da71d5f72"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="51bfcd92-eb3e-40f4-8778-2bbfb88a890b"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="cccaf3ac-2de9-44d4-aa31-54302fceb5f7"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>